<commit_message>
feat: add Story Map section (Day 5) with 7-beat documentary engine, 12-element worksheet, and direct pipeline bridge
</commit_message>
<xml_diff>
--- a/Pyschology and The Click (Completed).xlsx
+++ b/Pyschology and The Click (Completed).xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Audience Psychology &amp; The Click" sheetId="1" r:id="rId1"/>
+    <sheet name="Day 5 – Story Map" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,21 +399,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M11"/>
-  <cols>
-    <col min="1" max="1" width="6.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="55.83203125" customWidth="1"/>
-    <col min="7" max="7" width="45.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="50.83203125" customWidth="1"/>
-    <col min="10" max="10" width="50.83203125" customWidth="1"/>
-    <col min="11" max="11" width="50.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -940,4 +926,165 @@
     <ignoredError numberStoredAsText="1" sqref="A1:M11"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C13"/>
+  <cols>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="100.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>#</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Story Element</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Your Answer</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Working Title</v>
+      </c>
+      <c r="C2" t="str">
+        <v>How Did Ancient Egyptians Achieve Such Precise Stonework?</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Core Question</v>
+      </c>
+      <c r="C3" t="str">
+        <v>How did ancient Egyptian craftsmen shape, hollow, and align ultra-hard igneous rocks like granite, basalt, and diorite to sub-millimeter tolerances using Bronze Age copper tools and pounding stones without steel or powered machinery?</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Why Does It Matter?</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Hard igneous rocks like Aswan rose granite have a Mohs hardness of 6 to 7—harder than the copper and bronze tools available in the Bronze Age. Explaining how ancient builders overcame this material barrier proves the true height of human empirical engineering, directly dispelling pseudoscientific 'lost technology' claims.</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Cold Open</v>
+      </c>
+      <c r="C5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Visual: Extreme macro shot of a 12-pound spherical black diorite pounder striking crystalline pink granite in slow motion; fine quartz dust explodes into raking sunlight across a seam so tight no light passes through.
+Narration: 'This stone block was shaped more than 4,500 years ago. Its surface is remarkably flat, and its seams are so tight you cannot slide a razor blade between them.'</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Big Question</v>
+      </c>
+      <c r="C6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Visual: Pull back from the microscopic joint to reveal the colossal King's Chamber granite sarcophagus and unfinished obelisk in Aswan.
+Narration: 'Yet the people who carved it possessed no iron, no steel, and no diamond saws. So how did ancient Egyptian craftsmen achieve this level of precision with the tools available to them? To answer that, we have to look past the finished monuments and into the toolmarks left behind in the ancient quarries.'</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Context</v>
+      </c>
+      <c r="C7" t="str">
+        <v>During the Old and Middle Kingdoms (c. 2600–1800 BCE), Egyptian state projects quarried millions of tons of limestone and over 45,000 tons of hard igneous stone. Their metallurgy was limited to arsenical copper and bronze—alloys far softer than quartz crystals in granite. The dilemma is not whether they built it—the physical artifacts stand before us—but the exact physical mechanisms of material removal and precision measurement.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Investigation</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Experimental archaeologists, notably Denys Stocks and Mark Lehner, replicated ancient stonework techniques at Giza and Aswan. They systematically tested three distinct craft workflows: (1) heavy percussive fracturing using spherical dolerite pounders dropped from controlled heights, (2) tubular and flat saw cutting using copper blades fed with wet quartz sand abrasive slurry, and (3) precision surface dressing using flat wooden reference planes coated with red ochre pigment.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Complication</v>
+      </c>
+      <c r="C9" t="str">
+        <v>The Abrasive Paradox: Quartz sand has a Mohs hardness of 7—the exact same hardness as the quartz grains within the granite matrix. If the abrasive isn't harder than the stone, how could they saw massive sarcophagi without destroying tons of precious copper blades? Moreover, how were circular core drills stabilized without modern mechanical drill presses slipping across the convex rock face?</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Discovery / Evidence</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Scanning electron microscopy (SEM) of Petrie's famous drill core No. 7 and microscopic striations in unfinished quarry trenches revealed that the cutting was not done by copper teeth, but by quartz sand granules rolling and fracturing under immense downward pressure. The copper blade acted as a sacrificial carrier; the sharp angular quartz facets sheared microscopic mineral grains away. Furthermore, limestone guide blocks pinned to the rock face stabilized tubular drills.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Explanation</v>
+      </c>
+      <c r="C11" t="str">
+        <v>The precision was achieved not by high speed, but through continuous mechanical attrition and optical calibration: (1) dolerite pounding crushed crystalline bonds under impact, removing bulk rock; (2) copper blades and abrasive sand slurry sliced channels at roughly 12 cm³ per hour; and (3) surface flatness was measured using the 'three-rod method' with taut strings and red ochre rubbing blocks, iteratively grinding high spots down until total planar contact was achieved.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Final Payoff</v>
+      </c>
+      <c r="C12" t="str">
+        <v>The tight joints were not created by laser-like cutting, but by grinding matching stone faces against each other in situ with abrasive sand until they seated perfectly together. What appeared to be impossible engineering is revealed as an extraordinary mastery of physics, mineral friction, and organized craft labor repeated across generations.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Closing Thought</v>
+      </c>
+      <c r="C13" t="str">
+        <v>The true achievement of ancient Egyptian stonemasons is not that they possessed fantastical lost machinery, but that human patience, empirical observation of stone behavior, and communal dedication could transform raw geology into timeless precision using nothing more than rock, sand, and water.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C13"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(storymap): implement professional research discipline separating story idea, hypothesis, evidence, and verified narration for Egyptian stonework and AI engine
</commit_message>
<xml_diff>
--- a/Pyschology and The Click (Completed).xlsx
+++ b/Pyschology and The Click (Completed).xlsx
@@ -934,7 +934,7 @@
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="100.83203125" customWidth="1"/>
+    <col min="3" max="3" width="110.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -967,7 +967,7 @@
         <v>Core Question</v>
       </c>
       <c r="C3" t="str">
-        <v>How did ancient Egyptian craftsmen shape, hollow, and align ultra-hard igneous rocks like granite, basalt, and diorite to sub-millimeter tolerances using Bronze Age copper tools and pounding stones without steel or powered machinery?</v>
+        <v>How did ancient Egyptian craftsmen shape, hollow, and align ultra-hard igneous rocks like granite and basalt using Bronze Age copper tools and pounding stones without steel or powered machinery?</v>
       </c>
     </row>
     <row r="4">
@@ -978,7 +978,7 @@
         <v>Why Does It Matter?</v>
       </c>
       <c r="C4" t="str">
-        <v>Hard igneous rocks like Aswan rose granite have a Mohs hardness of 6 to 7—harder than the copper and bronze tools available in the Bronze Age. Explaining how ancient builders overcame this material barrier proves the true height of human empirical engineering, directly dispelling pseudoscientific 'lost technology' claims.</v>
+        <v>Hard igneous rocks like Aswan rose granite have a Mohs hardness of 6 to 7—harder than the copper tools available in the Bronze Age. Explaining how ancient builders overcame this material barrier proves the true height of human empirical engineering, directly dispelling pseudoscientific 'lost technology' claims.</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -989,8 +989,9 @@
         <v>Cold Open</v>
       </c>
       <c r="C5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Visual: Extreme macro shot of a 12-pound spherical black diorite pounder striking crystalline pink granite in slow motion; fine quartz dust explodes into raking sunlight across a seam so tight no light passes through.
-Narration: 'This stone block was shaped more than 4,500 years ago. Its surface is remarkably flat, and its seams are so tight you cannot slide a razor blade between them.'</v>
+        <v xml:space="preserve">Visual: Extreme macro shot of a heavy spherical dolerite pounder striking crystalline pink granite in slow motion; fine quartz dust explodes into raking sunlight across a tightly jointed megalithic seam.
+Narration: 'This stone block was shaped more than 4,500 years ago. Its surface is remarkably flat, and its seams are fitted with sub-millimeter precision.'
+[Needs research: (1) Verify museum weight distribution for Aswan dolerite mauls rather than asserting an exact 12-lb figure; (2) Cite Petrie's measured survey tolerances (~0.5mm mean joint) instead of the popular unverified 'razor blade cannot enter' trope.]</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -1002,62 +1003,67 @@
       </c>
       <c r="C6" t="str" xml:space="preserve">
         <v xml:space="preserve">Visual: Pull back from the microscopic joint to reveal the colossal King's Chamber granite sarcophagus and unfinished obelisk in Aswan.
-Narration: 'Yet the people who carved it possessed no iron, no steel, and no diamond saws. So how did ancient Egyptian craftsmen achieve this level of precision with the tools available to them? To answer that, we have to look past the finished monuments and into the toolmarks left behind in the ancient quarries.'</v>
-      </c>
-    </row>
-    <row r="7">
+Narration: 'Yet the people who carved it possessed no iron, no hardened steel, and no diamond saws. So how did ancient Egyptian craftsmen achieve this level of precision with the tools available to them? To answer that, we have to look past the finished monuments and into the toolmarks left behind in the ancient quarries.'</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="str">
         <v>Context</v>
       </c>
-      <c r="C7" t="str">
-        <v>During the Old and Middle Kingdoms (c. 2600–1800 BCE), Egyptian state projects quarried millions of tons of limestone and over 45,000 tons of hard igneous stone. Their metallurgy was limited to arsenical copper and bronze—alloys far softer than quartz crystals in granite. The dilemma is not whether they built it—the physical artifacts stand before us—but the exact physical mechanisms of material removal and precision measurement.</v>
-      </c>
-    </row>
-    <row r="8">
+      <c r="C7" t="str" xml:space="preserve">
+        <v xml:space="preserve">During the Old and Middle Kingdoms (c. 2600–1800 BCE), Egyptian state projects quarried millions of tons of limestone and thousands of tons of hard igneous stone. Their metallurgy was limited to arsenical copper and bronze—alloys far softer than quartz crystals in granite. The dilemma is not whether they built it—the physical artifacts stand before us—but the exact physical mechanisms of material removal and precision measurement.
+[Needs research: Verify primary archaeological and geological estimates for total Old Kingdom monumental granite tonnage quarried rather than citing an unverified 45,000-ton figure.]</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="str">
         <v>Investigation</v>
       </c>
-      <c r="C8" t="str">
-        <v>Experimental archaeologists, notably Denys Stocks and Mark Lehner, replicated ancient stonework techniques at Giza and Aswan. They systematically tested three distinct craft workflows: (1) heavy percussive fracturing using spherical dolerite pounders dropped from controlled heights, (2) tubular and flat saw cutting using copper blades fed with wet quartz sand abrasive slurry, and (3) precision surface dressing using flat wooden reference planes coated with red ochre pigment.</v>
-      </c>
-    </row>
-    <row r="9">
+      <c r="C8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Experimental archaeologists, notably Denys Stocks and Mark Lehner, replicated ancient stonework techniques at Giza and Aswan. They investigated three primary craft workflows: (1) percussive fracturing using spherical dolerite pounders, (2) tubular and flat saw cutting using copper blades fed with quartz sand abrasive slurry, and (3) surface dressing using reference planes and red ochre pigment.
+[Needs research: Distinguish documented physical tool finds (copper blades, dolerite balls, red-ochre marked stones) from modern experimental reconstructions to maintain evidence discipline.]</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="str">
         <v>Complication</v>
       </c>
-      <c r="C9" t="str">
-        <v>The Abrasive Paradox: Quartz sand has a Mohs hardness of 7—the exact same hardness as the quartz grains within the granite matrix. If the abrasive isn't harder than the stone, how could they saw massive sarcophagi without destroying tons of precious copper blades? Moreover, how were circular core drills stabilized without modern mechanical drill presses slipping across the convex rock face?</v>
-      </c>
-    </row>
-    <row r="10">
+      <c r="C9" t="str" xml:space="preserve">
+        <v xml:space="preserve">The Abrasive Paradox: Quartz sand has a Mohs hardness of 7—the same hardness as the quartz grains within the granite matrix. If the abrasive isn't harder than the stone, how could they saw massive sarcophagi without destroying immense amounts of precious copper? Moreover, how were circular core drills stabilized without modern mechanical drill presses slipping across the rock face?
+[Needs research: Determine whether archaeological evidence reveals a genuine recorded difficulty or if modern researchers are solving a problem ancient craft guilds handled through continuous lubrication and tool recycling.]</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="str">
         <v>Discovery / Evidence</v>
       </c>
-      <c r="C10" t="str">
-        <v>Scanning electron microscopy (SEM) of Petrie's famous drill core No. 7 and microscopic striations in unfinished quarry trenches revealed that the cutting was not done by copper teeth, but by quartz sand granules rolling and fracturing under immense downward pressure. The copper blade acted as a sacrificial carrier; the sharp angular quartz facets sheared microscopic mineral grains away. Furthermore, limestone guide blocks pinned to the rock face stabilized tubular drills.</v>
-      </c>
-    </row>
-    <row r="11">
+      <c r="C10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Microscopic striation analysis of Petrie's drill core No. 7 and unfinished quarry trenches suggests that cutting was facilitated by quartz sand granules rolling and micro-fracturing stone under heavy downward pressure, with the copper blade acting as a sacrificial carrier. Furthermore, researchers hypothesize that guide blocks were used to keep drill stems steady.
+[Needs research: (1) Review petrological debate regarding rolling vs embedded quartz-grain attrition in copper saw kerfs; (2) Verify whether physical limestone guide block artifacts have been excavated at Old Kingdom sites or if guide blocks remain an unconfirmed experimental hypothesis.]</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="str">
         <v>Explanation</v>
       </c>
-      <c r="C11" t="str">
-        <v>The precision was achieved not by high speed, but through continuous mechanical attrition and optical calibration: (1) dolerite pounding crushed crystalline bonds under impact, removing bulk rock; (2) copper blades and abrasive sand slurry sliced channels at roughly 12 cm³ per hour; and (3) surface flatness was measured using the 'three-rod method' with taut strings and red ochre rubbing blocks, iteratively grinding high spots down until total planar contact was achieved.</v>
+      <c r="C11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Modern experimental models suggest the precision was achieved through continuous mechanical attrition and optical calibration: (1) dolerite pounding crushed crystalline bonds under impact; (2) copper blades with abrasive slurry ground channels at rates documented by Stocks in modern tests; and (3) surface flatness was tested using red ochre rubbing blocks and hypothesized reference methods (such as the three-rod triangulation technique), grinding high spots until planar contact was achieved.
+[Needs research: (1) Cite Denys Stocks' specific experimental conditions for saw cutting rates (which varied widely by blade thickness, weight, and slurry) rather than stating '12 cm³/hr' as an absolute historical fact; (2) Cite primary evidence for workshop leveling techniques to determine whether the 'three-rod method' is attested in ancient Egyptian records or is an imported classical/modern masonry concept.]</v>
       </c>
     </row>
     <row r="12">
@@ -1068,7 +1074,7 @@
         <v>Final Payoff</v>
       </c>
       <c r="C12" t="str">
-        <v>The tight joints were not created by laser-like cutting, but by grinding matching stone faces against each other in situ with abrasive sand until they seated perfectly together. What appeared to be impossible engineering is revealed as an extraordinary mastery of physics, mineral friction, and organized craft labor repeated across generations.</v>
+        <v>The tight joints were not created by laser-like cutting, but by grinding matching stone faces against each other in situ with abrasive sand until they seated together. What appeared to be impossible engineering is revealed as an extraordinary mastery of physics, mineral friction, and organized craft labor repeated across generations.</v>
       </c>
     </row>
     <row r="13">

</xml_diff>